<commit_message>
Refresh ESPN and Yahoo adjusted rankings
</commit_message>
<xml_diff>
--- a/frontend/public/data/2026/espn/merged_formatted.xlsx
+++ b/frontend/public/data/2026/espn/merged_formatted.xlsx
@@ -616,7 +616,7 @@
         <v>55</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>4</v>
@@ -651,7 +651,7 @@
         <v>56</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>3</v>
@@ -791,7 +791,7 @@
         <v>52</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>5</v>
@@ -826,7 +826,7 @@
         <v>54</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>8</v>
@@ -1771,7 +1771,7 @@
         <v>21</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>27</v>
@@ -1806,7 +1806,7 @@
         <v>23</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>38</v>
@@ -1841,7 +1841,7 @@
         <v>25</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>35</v>
@@ -2261,7 +2261,7 @@
         <v>10</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I50" s="3" t="n">
         <v>56</v>
@@ -2296,7 +2296,7 @@
         <v>8</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I51" s="3" t="n">
         <v>53</v>
@@ -2366,7 +2366,7 @@
         <v>6</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I53" s="3" t="n">
         <v>59</v>
@@ -2401,7 +2401,7 @@
         <v>17</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I54" s="3" t="n">
         <v>45</v>
@@ -2436,7 +2436,7 @@
         <v>13</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I55" s="3" t="n">
         <v>46</v>
@@ -2471,7 +2471,7 @@
         <v>5</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I56" s="3" t="n">
         <v>68</v>
@@ -2541,7 +2541,7 @@
         <v>10</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I58" s="3" t="n">
         <v>58</v>
@@ -2576,7 +2576,7 @@
         <v>9</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I59" s="3" t="n">
         <v>57</v>
@@ -2611,7 +2611,7 @@
         <v>14</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I60" s="3" t="n">
         <v>50</v>
@@ -2646,7 +2646,7 @@
         <v>4</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I61" s="3" t="n">
         <v>71</v>
@@ -2681,7 +2681,7 @@
         <v>3</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I62" s="3" t="n">
         <v>83</v>
@@ -2751,7 +2751,7 @@
         <v>9</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I64" s="3" t="n">
         <v>73</v>
@@ -2786,7 +2786,7 @@
         <v>6</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I65" s="3" t="n">
         <v>61</v>
@@ -2821,7 +2821,7 @@
         <v>7</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I66" s="3" t="n">
         <v>66</v>
@@ -2891,7 +2891,7 @@
         <v>2</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I68" s="3" t="n">
         <v>120</v>
@@ -2926,7 +2926,7 @@
         <v>3</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I69" s="3" t="n">
         <v>86</v>
@@ -2961,7 +2961,7 @@
         <v>5</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I70" s="3" t="n">
         <v>89</v>
@@ -2996,7 +2996,7 @@
         <v>9</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I71" s="3" t="n">
         <v>79</v>
@@ -3031,7 +3031,7 @@
         <v>6</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I72" s="3" t="n">
         <v>77</v>
@@ -3066,7 +3066,7 @@
         <v>2</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I73" s="3" t="n">
         <v>105</v>
@@ -3101,7 +3101,7 @@
         <v>3</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I74" s="3" t="n">
         <v>94</v>
@@ -3171,7 +3171,7 @@
         <v>3</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I76" s="3" t="n">
         <v>70</v>
@@ -3206,7 +3206,7 @@
         <v>17</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I77" s="3" t="n">
         <v>44</v>
@@ -3241,7 +3241,7 @@
         <v>7</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I78" s="3" t="n">
         <v>64</v>
@@ -3311,7 +3311,7 @@
         <v>2</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I80" s="3" t="n">
         <v>129</v>
@@ -3346,7 +3346,7 @@
         <v>1</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="I81" s="3" t="n">
         <v>113</v>
@@ -3381,7 +3381,7 @@
         <v>7</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I82" s="3" t="n">
         <v>63</v>
@@ -3416,7 +3416,7 @@
         <v>4</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I83" s="3" t="n">
         <v>97</v>
@@ -3451,7 +3451,7 @@
         <v>2</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="I84" s="3" t="n">
         <v>91</v>
@@ -3521,7 +3521,7 @@
         <v>3</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I86" s="3" t="n">
         <v>88</v>
@@ -3556,7 +3556,7 @@
         <v>2</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="I87" s="3" t="n">
         <v>108</v>
@@ -3591,7 +3591,7 @@
         <v>4</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="I88" s="3" t="n">
         <v>69</v>
@@ -3661,7 +3661,7 @@
         <v>3</v>
       </c>
       <c r="H90" s="3" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="I90" s="3" t="n">
         <v>110</v>
@@ -3696,7 +3696,7 @@
         <v>7</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I91" s="3" t="n">
         <v>75</v>
@@ -3731,7 +3731,7 @@
         <v>5</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I92" s="3" t="n">
         <v>80</v>
@@ -3766,7 +3766,7 @@
         <v>4</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I93" s="3" t="n">
         <v>85</v>
@@ -3836,7 +3836,7 @@
         <v>2</v>
       </c>
       <c r="H95" s="3" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I95" s="3" t="n">
         <v>93</v>
@@ -3871,7 +3871,7 @@
         <v>2</v>
       </c>
       <c r="H96" s="3" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I96" s="3" t="n">
         <v>124</v>
@@ -3906,7 +3906,7 @@
         <v>11</v>
       </c>
       <c r="H97" s="3" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I97" s="3" t="n">
         <v>72</v>
@@ -3941,7 +3941,7 @@
         <v>1</v>
       </c>
       <c r="H98" s="3" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="I98" s="3" t="n">
         <v>103</v>
@@ -3976,7 +3976,7 @@
         <v>2</v>
       </c>
       <c r="H99" s="3" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="I99" s="3" t="n">
         <v>114</v>
@@ -4011,7 +4011,7 @@
         <v>2</v>
       </c>
       <c r="H100" s="3" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I100" s="3" t="n">
         <v>84</v>
@@ -4046,7 +4046,7 @@
         <v>1</v>
       </c>
       <c r="H101" s="3" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I101" s="3" t="n">
         <v>130</v>
@@ -4081,7 +4081,7 @@
         <v>2</v>
       </c>
       <c r="H102" s="3" t="n">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I102" s="3" t="n">
         <v>121</v>
@@ -4116,7 +4116,7 @@
         <v>5</v>
       </c>
       <c r="H103" s="3" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="I103" s="3" t="n">
         <v>74</v>
@@ -4151,7 +4151,7 @@
         <v>3</v>
       </c>
       <c r="H104" s="3" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I104" s="3" t="n">
         <v>98</v>
@@ -4186,7 +4186,7 @@
         <v>3</v>
       </c>
       <c r="H105" s="3" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I105" s="3" t="n">
         <v>76</v>
@@ -4221,7 +4221,7 @@
         <v>4</v>
       </c>
       <c r="H106" s="3" t="n">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I106" s="3" t="n">
         <v>96</v>
@@ -4256,7 +4256,7 @@
         <v>2</v>
       </c>
       <c r="H107" s="3" t="n">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="I107" s="3" t="n">
         <v>127</v>
@@ -4291,7 +4291,7 @@
         <v>2</v>
       </c>
       <c r="H108" s="3" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="I108" s="3" t="n">
         <v>122</v>
@@ -4326,7 +4326,7 @@
         <v>1</v>
       </c>
       <c r="H109" s="3" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I109" s="3" t="n">
         <v>131</v>
@@ -4361,7 +4361,7 @@
         <v>1</v>
       </c>
       <c r="H110" s="3" t="n">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="I110" s="3" t="n">
         <v>150</v>
@@ -4396,7 +4396,7 @@
         <v>2</v>
       </c>
       <c r="H111" s="3" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="I111" s="3" t="n">
         <v>90</v>
@@ -4431,7 +4431,7 @@
         <v>2</v>
       </c>
       <c r="H112" s="3" t="n">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="I112" s="3" t="n">
         <v>92</v>
@@ -4466,7 +4466,7 @@
         <v>1</v>
       </c>
       <c r="H113" s="3" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="I113" s="3" t="n">
         <v>102</v>
@@ -4501,7 +4501,7 @@
         <v>1</v>
       </c>
       <c r="H114" s="3" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I114" s="3" t="n">
         <v>158</v>
@@ -4536,7 +4536,7 @@
         <v>4</v>
       </c>
       <c r="H115" s="3" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="I115" s="3" t="n">
         <v>82</v>
@@ -4571,7 +4571,7 @@
         <v>2</v>
       </c>
       <c r="H116" s="3" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I116" s="3" t="n">
         <v>106</v>
@@ -4606,7 +4606,7 @@
         <v>4</v>
       </c>
       <c r="H117" s="3" t="n">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="I117" s="3" t="n">
         <v>78</v>
@@ -4641,7 +4641,7 @@
         <v>2</v>
       </c>
       <c r="H118" s="3" t="n">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="I118" s="3" t="n">
         <v>99</v>
@@ -4676,7 +4676,7 @@
         <v>4</v>
       </c>
       <c r="H119" s="3" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I119" s="3" t="n">
         <v>95</v>
@@ -4711,7 +4711,7 @@
         <v>1</v>
       </c>
       <c r="H120" s="3" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I120" s="3" t="n">
         <v>144</v>
@@ -4746,7 +4746,7 @@
         <v>3</v>
       </c>
       <c r="H121" s="3" t="n">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="I121" s="3" t="n">
         <v>109</v>
@@ -4781,7 +4781,7 @@
         <v>1</v>
       </c>
       <c r="H122" s="3" t="n">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="I122" s="3" t="n">
         <v>101</v>
@@ -4816,7 +4816,7 @@
         <v>2</v>
       </c>
       <c r="H123" s="3" t="n">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="I123" s="3" t="n">
         <v>118</v>
@@ -4851,7 +4851,7 @@
         <v>2</v>
       </c>
       <c r="H124" s="3" t="n">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="I124" s="3" t="n">
         <v>119</v>
@@ -4886,7 +4886,7 @@
         <v>2</v>
       </c>
       <c r="H125" s="3" t="n">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="I125" s="3" t="n">
         <v>133</v>
@@ -4921,7 +4921,7 @@
         <v>4</v>
       </c>
       <c r="H126" s="3" t="n">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="I126" s="3" t="n">
         <v>104</v>
@@ -4956,7 +4956,7 @@
         <v>0</v>
       </c>
       <c r="H127" s="3" t="n">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="I127" s="3" t="n">
         <v>147</v>
@@ -4991,7 +4991,7 @@
         <v>0</v>
       </c>
       <c r="H128" s="3" t="n">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="I128" s="3" t="n">
         <v>164</v>
@@ -5026,7 +5026,7 @@
         <v>1</v>
       </c>
       <c r="H129" s="3" t="n">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="I129" s="3" t="n">
         <v>128</v>
@@ -5096,7 +5096,7 @@
         <v>1</v>
       </c>
       <c r="H131" s="3" t="n">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="I131" s="3" t="n">
         <v>112</v>
@@ -5131,7 +5131,7 @@
         <v>1</v>
       </c>
       <c r="H132" s="3" t="n">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="I132" s="3" t="n">
         <v>123</v>
@@ -5166,7 +5166,7 @@
         <v>6</v>
       </c>
       <c r="H133" s="3" t="n">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="I133" s="3" t="n">
         <v>81</v>
@@ -5201,7 +5201,7 @@
         <v>0</v>
       </c>
       <c r="H134" s="3" t="n">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="I134" s="3" t="n">
         <v>168</v>
@@ -5236,7 +5236,7 @@
         <v>0</v>
       </c>
       <c r="H135" s="3" t="n">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I135" s="3" t="inlineStr"/>
     </row>
@@ -5304,7 +5304,7 @@
         <v>0</v>
       </c>
       <c r="H137" s="3" t="n">
-        <v>168</v>
+        <v>258</v>
       </c>
       <c r="I137" s="3" t="n">
         <v>263</v>
@@ -5339,7 +5339,7 @@
         <v>1</v>
       </c>
       <c r="H138" s="3" t="n">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="I138" s="3" t="n">
         <v>132</v>
@@ -5374,7 +5374,7 @@
         <v>0</v>
       </c>
       <c r="H139" s="3" t="n">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="I139" s="3" t="n">
         <v>186</v>
@@ -5409,7 +5409,7 @@
         <v>2</v>
       </c>
       <c r="H140" s="3" t="n">
-        <v>207</v>
+        <v>147</v>
       </c>
       <c r="I140" s="3" t="n">
         <v>107</v>
@@ -5444,7 +5444,7 @@
         <v>0</v>
       </c>
       <c r="H141" s="3" t="n">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="I141" s="3" t="n">
         <v>197</v>
@@ -5479,7 +5479,7 @@
         <v>2</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="I142" s="3" t="n">
         <v>143</v>
@@ -5514,7 +5514,7 @@
         <v>0</v>
       </c>
       <c r="H143" s="3" t="n">
-        <v>240</v>
+        <v>224</v>
       </c>
       <c r="I143" s="3" t="n">
         <v>236</v>
@@ -5549,7 +5549,7 @@
         <v>0</v>
       </c>
       <c r="H144" s="3" t="n">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="I144" s="3" t="n">
         <v>163</v>
@@ -5584,7 +5584,7 @@
         <v>0</v>
       </c>
       <c r="H145" s="3" t="n">
-        <v>210</v>
+        <v>194</v>
       </c>
       <c r="I145" s="3" t="n">
         <v>185</v>
@@ -5619,7 +5619,7 @@
         <v>2</v>
       </c>
       <c r="H146" s="3" t="n">
-        <v>187</v>
+        <v>148</v>
       </c>
       <c r="I146" s="3" t="n">
         <v>115</v>
@@ -5654,7 +5654,7 @@
         <v>0</v>
       </c>
       <c r="H147" s="3" t="n">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="I147" s="3" t="n">
         <v>193</v>
@@ -5689,7 +5689,7 @@
         <v>0</v>
       </c>
       <c r="H148" s="3" t="n">
-        <v>218</v>
+        <v>202</v>
       </c>
       <c r="I148" s="3" t="n">
         <v>200</v>
@@ -5724,7 +5724,7 @@
         <v>0</v>
       </c>
       <c r="H149" s="3" t="n">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="I149" s="3" t="n">
         <v>145</v>
@@ -5759,7 +5759,7 @@
         <v>1</v>
       </c>
       <c r="H150" s="3" t="n">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="I150" s="3" t="n">
         <v>152</v>
@@ -5794,7 +5794,7 @@
         <v>0</v>
       </c>
       <c r="H151" s="3" t="n">
-        <v>243</v>
+        <v>227</v>
       </c>
       <c r="I151" s="3" t="n">
         <v>239</v>
@@ -5829,7 +5829,7 @@
         <v>1</v>
       </c>
       <c r="H152" s="3" t="n">
-        <v>208</v>
+        <v>146</v>
       </c>
       <c r="I152" s="3" t="n">
         <v>111</v>
@@ -5864,7 +5864,7 @@
         <v>0</v>
       </c>
       <c r="H153" s="3" t="n">
-        <v>205</v>
+        <v>189</v>
       </c>
       <c r="I153" s="3" t="n">
         <v>170</v>
@@ -5899,7 +5899,7 @@
         <v>1</v>
       </c>
       <c r="H154" s="3" t="n">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="I154" s="3" t="n">
         <v>160</v>
@@ -5934,7 +5934,7 @@
         <v>1</v>
       </c>
       <c r="H155" s="3" t="n">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="I155" s="3" t="n">
         <v>135</v>
@@ -5969,7 +5969,7 @@
         <v>1</v>
       </c>
       <c r="H156" s="3" t="n">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="I156" s="3" t="n">
         <v>149</v>
@@ -6004,7 +6004,7 @@
         <v>0</v>
       </c>
       <c r="H157" s="3" t="n">
-        <v>228</v>
+        <v>212</v>
       </c>
       <c r="I157" s="3" t="n">
         <v>218</v>
@@ -6039,7 +6039,7 @@
         <v>0</v>
       </c>
       <c r="H158" s="3" t="n">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="I158" s="3" t="n">
         <v>232</v>
@@ -6074,7 +6074,7 @@
         <v>0</v>
       </c>
       <c r="H159" s="3" t="n">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="I159" s="3" t="n">
         <v>173</v>
@@ -6109,7 +6109,7 @@
         <v>1</v>
       </c>
       <c r="H160" s="3" t="n">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="I160" s="3" t="n">
         <v>167</v>
@@ -6144,7 +6144,7 @@
         <v>0</v>
       </c>
       <c r="H161" s="3" t="n">
-        <v>246</v>
+        <v>230</v>
       </c>
       <c r="I161" s="3" t="n">
         <v>221</v>
@@ -6179,7 +6179,7 @@
         <v>0</v>
       </c>
       <c r="H162" s="3" t="n">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="I162" s="3" t="n">
         <v>142</v>
@@ -6214,7 +6214,7 @@
         <v>1</v>
       </c>
       <c r="H163" s="3" t="n">
-        <v>209</v>
+        <v>149</v>
       </c>
       <c r="I163" s="3" t="n">
         <v>134</v>
@@ -6249,7 +6249,7 @@
         <v>1</v>
       </c>
       <c r="H164" s="3" t="n">
-        <v>186</v>
+        <v>209</v>
       </c>
       <c r="I164" s="3" t="n">
         <v>136</v>
@@ -6284,7 +6284,7 @@
         <v>0</v>
       </c>
       <c r="H165" s="3" t="n">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="I165" s="3" t="n">
         <v>220</v>
@@ -6319,7 +6319,7 @@
         <v>0</v>
       </c>
       <c r="H166" s="3" t="n">
-        <v>212</v>
+        <v>196</v>
       </c>
       <c r="I166" s="3" t="n">
         <v>177</v>
@@ -6354,7 +6354,7 @@
         <v>0</v>
       </c>
       <c r="H167" s="3" t="n">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="I167" s="3" t="n">
         <v>146</v>
@@ -6389,7 +6389,7 @@
         <v>0</v>
       </c>
       <c r="H168" s="3" t="n">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="I168" s="3" t="n">
         <v>201</v>
@@ -6424,7 +6424,7 @@
         <v>0</v>
       </c>
       <c r="H169" s="3" t="n">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="I169" s="3" t="n">
         <v>223</v>
@@ -6459,7 +6459,7 @@
         <v>0</v>
       </c>
       <c r="H170" s="3" t="n">
-        <v>195</v>
+        <v>179</v>
       </c>
       <c r="I170" s="3" t="n">
         <v>172</v>
@@ -6494,7 +6494,7 @@
         <v>0</v>
       </c>
       <c r="H171" s="3" t="n">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="I171" s="3" t="n">
         <v>219</v>
@@ -6529,7 +6529,7 @@
         <v>0</v>
       </c>
       <c r="H172" s="3" t="n">
-        <v>249</v>
+        <v>233</v>
       </c>
       <c r="I172" s="3" t="n">
         <v>228</v>
@@ -6564,7 +6564,7 @@
         <v>0</v>
       </c>
       <c r="H173" s="3" t="n">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="I173" s="3" t="n">
         <v>169</v>
@@ -6599,7 +6599,7 @@
         <v>0</v>
       </c>
       <c r="H174" s="3" t="n">
-        <v>161</v>
+        <v>245</v>
       </c>
       <c r="I174" s="3" t="n">
         <v>238</v>
@@ -6634,7 +6634,7 @@
         <v>1</v>
       </c>
       <c r="H175" s="3" t="n">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="I175" s="3" t="n">
         <v>117</v>
@@ -6704,7 +6704,7 @@
         <v>0</v>
       </c>
       <c r="H177" s="3" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="I177" s="3" t="n">
         <v>140</v>
@@ -6739,7 +6739,7 @@
         <v>0</v>
       </c>
       <c r="H178" s="3" t="n">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="I178" s="3" t="n">
         <v>206</v>
@@ -6774,7 +6774,7 @@
         <v>1</v>
       </c>
       <c r="H179" s="3" t="n">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="I179" s="3" t="n">
         <v>116</v>
@@ -6809,7 +6809,7 @@
         <v>0</v>
       </c>
       <c r="H180" s="3" t="n">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="I180" s="3" t="n">
         <v>183</v>
@@ -6844,7 +6844,7 @@
         <v>0</v>
       </c>
       <c r="H181" s="3" t="n">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="I181" s="3" t="n">
         <v>298</v>
@@ -6879,7 +6879,7 @@
         <v>0</v>
       </c>
       <c r="H182" s="3" t="n">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="I182" s="3" t="n">
         <v>156</v>
@@ -6914,7 +6914,7 @@
         <v>0</v>
       </c>
       <c r="H183" s="3" t="n">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="I183" s="3" t="n">
         <v>196</v>
@@ -6949,7 +6949,7 @@
         <v>0</v>
       </c>
       <c r="H184" s="3" t="n">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="I184" s="3" t="n">
         <v>157</v>
@@ -6984,7 +6984,7 @@
         <v>0</v>
       </c>
       <c r="H185" s="3" t="n">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="I185" s="3" t="n">
         <v>181</v>
@@ -7019,7 +7019,7 @@
         <v>0</v>
       </c>
       <c r="H186" s="3" t="n">
-        <v>194</v>
+        <v>178</v>
       </c>
       <c r="I186" s="3" t="n">
         <v>161</v>
@@ -7054,7 +7054,7 @@
         <v>0</v>
       </c>
       <c r="H187" s="3" t="n">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="I187" s="3" t="n">
         <v>192</v>
@@ -7089,7 +7089,7 @@
         <v>0</v>
       </c>
       <c r="H188" s="3" t="n">
-        <v>152</v>
+        <v>243</v>
       </c>
       <c r="I188" s="3" t="n">
         <v>264</v>
@@ -7124,7 +7124,7 @@
         <v>0</v>
       </c>
       <c r="H189" s="3" t="n">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="I189" s="3" t="n">
         <v>210</v>
@@ -7159,7 +7159,7 @@
         <v>1</v>
       </c>
       <c r="H190" s="3" t="n">
-        <v>184</v>
+        <v>168</v>
       </c>
       <c r="I190" s="3" t="n">
         <v>151</v>
@@ -7194,7 +7194,7 @@
         <v>0</v>
       </c>
       <c r="H191" s="3" t="n">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="I191" s="3" t="n">
         <v>166</v>
@@ -7229,7 +7229,7 @@
         <v>0</v>
       </c>
       <c r="H192" s="3" t="n">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="I192" s="3" t="n">
         <v>165</v>
@@ -7264,7 +7264,7 @@
         <v>0</v>
       </c>
       <c r="H193" s="3" t="n">
-        <v>256</v>
+        <v>240</v>
       </c>
       <c r="I193" s="3" t="n">
         <v>231</v>
@@ -7299,7 +7299,7 @@
         <v>0</v>
       </c>
       <c r="H194" s="3" t="n">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="I194" s="3" t="n">
         <v>222</v>
@@ -7334,7 +7334,7 @@
         <v>0</v>
       </c>
       <c r="H195" s="3" t="n">
-        <v>227</v>
+        <v>213</v>
       </c>
       <c r="I195" s="3" t="n">
         <v>246</v>
@@ -7369,7 +7369,7 @@
         <v>0</v>
       </c>
       <c r="H196" s="3" t="n">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="I196" s="3" t="n">
         <v>217</v>
@@ -7404,7 +7404,7 @@
         <v>0</v>
       </c>
       <c r="H197" s="3" t="n">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="I197" s="3" t="n">
         <v>202</v>
@@ -7439,7 +7439,7 @@
         <v>1</v>
       </c>
       <c r="H198" s="3" t="n">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="I198" s="3" t="n">
         <v>159</v>
@@ -7474,7 +7474,7 @@
         <v>0</v>
       </c>
       <c r="H199" s="3" t="n">
-        <v>166</v>
+        <v>256</v>
       </c>
       <c r="I199" s="3" t="n">
         <v>247</v>
@@ -7509,7 +7509,7 @@
         <v>0</v>
       </c>
       <c r="H200" s="3" t="n">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="I200" s="3" t="n">
         <v>174</v>
@@ -7544,7 +7544,7 @@
         <v>0</v>
       </c>
       <c r="H201" s="3" t="n">
-        <v>196</v>
+        <v>180</v>
       </c>
       <c r="I201" s="3" t="n">
         <v>175</v>
@@ -7579,7 +7579,7 @@
         <v>0</v>
       </c>
       <c r="H202" s="3" t="n">
-        <v>239</v>
+        <v>223</v>
       </c>
       <c r="I202" s="3" t="n">
         <v>248</v>
@@ -7614,7 +7614,7 @@
         <v>0</v>
       </c>
       <c r="H203" s="3" t="n">
-        <v>150</v>
+        <v>268</v>
       </c>
       <c r="I203" s="3" t="n">
         <v>278</v>
@@ -7649,7 +7649,7 @@
         <v>0</v>
       </c>
       <c r="H204" s="3" t="n">
-        <v>167</v>
+        <v>257</v>
       </c>
       <c r="I204" s="3" t="n">
         <v>262</v>
@@ -7684,7 +7684,7 @@
         <v>0</v>
       </c>
       <c r="H205" s="3" t="n">
-        <v>259</v>
+        <v>162</v>
       </c>
       <c r="I205" s="3" t="n">
         <v>288</v>
@@ -7719,7 +7719,7 @@
         <v>0</v>
       </c>
       <c r="H206" s="3" t="n">
-        <v>160</v>
+        <v>251</v>
       </c>
       <c r="I206" s="3" t="n">
         <v>266</v>
@@ -7754,7 +7754,7 @@
         <v>0</v>
       </c>
       <c r="H207" s="3" t="n">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="I207" s="3" t="n">
         <v>188</v>
@@ -7789,7 +7789,7 @@
         <v>0</v>
       </c>
       <c r="H208" s="3" t="n">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="I208" s="3" t="n">
         <v>187</v>
@@ -7824,7 +7824,7 @@
         <v>0</v>
       </c>
       <c r="H209" s="3" t="n">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="I209" s="3" t="n">
         <v>198</v>
@@ -7859,7 +7859,7 @@
         <v>0</v>
       </c>
       <c r="H210" s="3" t="n">
-        <v>244</v>
+        <v>228</v>
       </c>
       <c r="I210" s="3" t="n">
         <v>215</v>
@@ -7894,7 +7894,7 @@
         <v>0</v>
       </c>
       <c r="H211" s="3" t="n">
-        <v>254</v>
+        <v>238</v>
       </c>
       <c r="I211" s="3" t="n">
         <v>249</v>
@@ -7929,7 +7929,7 @@
         <v>0</v>
       </c>
       <c r="H212" s="3" t="n">
-        <v>147</v>
+        <v>269</v>
       </c>
       <c r="I212" s="3" t="n">
         <v>300</v>
@@ -7964,7 +7964,7 @@
         <v>0</v>
       </c>
       <c r="H213" s="3" t="n">
-        <v>169</v>
+        <v>259</v>
       </c>
       <c r="I213" s="3" t="n">
         <v>292</v>
@@ -7999,7 +7999,7 @@
         <v>0</v>
       </c>
       <c r="H214" s="3" t="n">
-        <v>163</v>
+        <v>253</v>
       </c>
       <c r="I214" s="3" t="n">
         <v>250</v>
@@ -8034,7 +8034,7 @@
         <v>0</v>
       </c>
       <c r="H215" s="3" t="n">
-        <v>263</v>
+        <v>154</v>
       </c>
       <c r="I215" s="3" t="inlineStr"/>
     </row>
@@ -8067,7 +8067,7 @@
         <v>0</v>
       </c>
       <c r="H216" s="3" t="n">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="I216" s="3" t="n">
         <v>178</v>
@@ -8102,7 +8102,7 @@
         <v>0</v>
       </c>
       <c r="H217" s="3" t="n">
-        <v>261</v>
+        <v>166</v>
       </c>
       <c r="I217" s="3" t="n">
         <v>294</v>
@@ -8137,7 +8137,7 @@
         <v>0</v>
       </c>
       <c r="H218" s="3" t="n">
-        <v>162</v>
+        <v>252</v>
       </c>
       <c r="I218" s="3" t="n">
         <v>245</v>
@@ -8172,7 +8172,7 @@
         <v>0</v>
       </c>
       <c r="H219" s="3" t="n">
-        <v>164</v>
+        <v>254</v>
       </c>
       <c r="I219" s="3" t="n">
         <v>276</v>
@@ -8207,7 +8207,7 @@
         <v>0</v>
       </c>
       <c r="H220" s="3" t="n">
-        <v>271</v>
+        <v>152</v>
       </c>
       <c r="I220" s="3" t="inlineStr"/>
     </row>
@@ -8240,7 +8240,7 @@
         <v>0</v>
       </c>
       <c r="H221" s="3" t="n">
-        <v>202</v>
+        <v>186</v>
       </c>
       <c r="I221" s="3" t="n">
         <v>176</v>
@@ -8275,7 +8275,7 @@
         <v>0</v>
       </c>
       <c r="H222" s="3" t="n">
-        <v>175</v>
+        <v>265</v>
       </c>
       <c r="I222" s="3" t="inlineStr"/>
     </row>
@@ -8308,7 +8308,7 @@
         <v>0</v>
       </c>
       <c r="H223" s="3" t="n">
-        <v>154</v>
+        <v>244</v>
       </c>
       <c r="I223" s="3" t="inlineStr"/>
     </row>
@@ -8341,7 +8341,7 @@
         <v>0</v>
       </c>
       <c r="H224" s="3" t="n">
-        <v>237</v>
+        <v>221</v>
       </c>
       <c r="I224" s="3" t="n">
         <v>275</v>
@@ -8376,7 +8376,7 @@
         <v>0</v>
       </c>
       <c r="H225" s="3" t="n">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="I225" s="3" t="n">
         <v>240</v>
@@ -8411,7 +8411,7 @@
         <v>0</v>
       </c>
       <c r="H226" s="3" t="n">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="I226" s="3" t="n">
         <v>224</v>
@@ -8446,7 +8446,7 @@
         <v>0</v>
       </c>
       <c r="H227" s="3" t="n">
-        <v>206</v>
+        <v>190</v>
       </c>
       <c r="I227" s="3" t="n">
         <v>209</v>
@@ -8481,7 +8481,7 @@
         <v>0</v>
       </c>
       <c r="H228" s="3" t="n">
-        <v>172</v>
+        <v>262</v>
       </c>
       <c r="I228" s="3" t="n">
         <v>291</v>
@@ -8516,7 +8516,7 @@
         <v>0</v>
       </c>
       <c r="H229" s="3" t="n">
-        <v>269</v>
+        <v>160</v>
       </c>
       <c r="I229" s="3" t="inlineStr"/>
     </row>
@@ -8549,7 +8549,7 @@
         <v>0</v>
       </c>
       <c r="H230" s="3" t="n">
-        <v>148</v>
+        <v>270</v>
       </c>
       <c r="I230" s="3" t="n">
         <v>284</v>
@@ -8584,7 +8584,7 @@
         <v>0</v>
       </c>
       <c r="H231" s="3" t="n">
-        <v>151</v>
+        <v>271</v>
       </c>
       <c r="I231" s="3" t="n">
         <v>279</v>
@@ -8619,7 +8619,7 @@
         <v>0</v>
       </c>
       <c r="H232" s="3" t="n">
-        <v>257</v>
+        <v>164</v>
       </c>
       <c r="I232" s="3" t="n">
         <v>286</v>
@@ -8654,7 +8654,7 @@
         <v>0</v>
       </c>
       <c r="H233" s="3" t="n">
-        <v>232</v>
+        <v>216</v>
       </c>
       <c r="I233" s="3" t="n">
         <v>252</v>
@@ -8689,7 +8689,7 @@
         <v>0</v>
       </c>
       <c r="H234" s="3" t="n">
-        <v>153</v>
+        <v>242</v>
       </c>
       <c r="I234" s="3" t="n">
         <v>237</v>
@@ -8724,7 +8724,7 @@
         <v>0</v>
       </c>
       <c r="H235" s="3" t="n">
-        <v>149</v>
+        <v>272</v>
       </c>
       <c r="I235" s="3" t="n">
         <v>285</v>
@@ -8759,7 +8759,7 @@
         <v>0</v>
       </c>
       <c r="H236" s="3" t="n">
-        <v>155</v>
+        <v>249</v>
       </c>
       <c r="I236" s="3" t="n">
         <v>289</v>
@@ -8794,7 +8794,7 @@
         <v>0</v>
       </c>
       <c r="H237" s="3" t="n">
-        <v>272</v>
+        <v>151</v>
       </c>
       <c r="I237" s="3" t="n">
         <v>290</v>
@@ -8829,7 +8829,7 @@
         <v>0</v>
       </c>
       <c r="H238" s="3" t="n">
-        <v>247</v>
+        <v>231</v>
       </c>
       <c r="I238" s="3" t="n">
         <v>229</v>
@@ -8864,7 +8864,7 @@
         <v>0</v>
       </c>
       <c r="H239" s="3" t="n">
-        <v>165</v>
+        <v>255</v>
       </c>
       <c r="I239" s="3" t="n">
         <v>244</v>
@@ -8899,7 +8899,7 @@
         <v>0</v>
       </c>
       <c r="H240" s="3" t="n">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="I240" s="3" t="n">
         <v>182</v>
@@ -8934,7 +8934,7 @@
         <v>0</v>
       </c>
       <c r="H241" s="3" t="n">
-        <v>156</v>
+        <v>246</v>
       </c>
       <c r="I241" s="3" t="inlineStr"/>
     </row>
@@ -8967,7 +8967,7 @@
         <v>0</v>
       </c>
       <c r="H242" s="3" t="n">
-        <v>234</v>
+        <v>218</v>
       </c>
       <c r="I242" s="3" t="n">
         <v>205</v>
@@ -9002,7 +9002,7 @@
         <v>0</v>
       </c>
       <c r="H243" s="3" t="n">
-        <v>235</v>
+        <v>219</v>
       </c>
       <c r="I243" s="3" t="n">
         <v>204</v>
@@ -9037,7 +9037,7 @@
         <v>0</v>
       </c>
       <c r="H244" s="3" t="n">
-        <v>253</v>
+        <v>237</v>
       </c>
       <c r="I244" s="3" t="n">
         <v>243</v>
@@ -9072,7 +9072,7 @@
         <v>0</v>
       </c>
       <c r="H245" s="3" t="n">
-        <v>203</v>
+        <v>187</v>
       </c>
       <c r="I245" s="3" t="n">
         <v>191</v>
@@ -9107,7 +9107,7 @@
         <v>0</v>
       </c>
       <c r="H246" s="3" t="n">
-        <v>264</v>
+        <v>155</v>
       </c>
       <c r="I246" s="3" t="n">
         <v>296</v>
@@ -9142,7 +9142,7 @@
         <v>0</v>
       </c>
       <c r="H247" s="3" t="n">
-        <v>248</v>
+        <v>232</v>
       </c>
       <c r="I247" s="3" t="n">
         <v>273</v>
@@ -9212,7 +9212,7 @@
         <v>0</v>
       </c>
       <c r="H249" s="3" t="n">
-        <v>251</v>
+        <v>235</v>
       </c>
       <c r="I249" s="3" t="n">
         <v>299</v>
@@ -9247,7 +9247,7 @@
         <v>0</v>
       </c>
       <c r="H250" s="3" t="n">
-        <v>231</v>
+        <v>215</v>
       </c>
       <c r="I250" s="3" t="n">
         <v>214</v>
@@ -9282,7 +9282,7 @@
         <v>0</v>
       </c>
       <c r="H251" s="3" t="n">
-        <v>230</v>
+        <v>214</v>
       </c>
       <c r="I251" s="3" t="n">
         <v>199</v>
@@ -9317,7 +9317,7 @@
         <v>0</v>
       </c>
       <c r="H252" s="3" t="n">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="I252" s="3" t="n">
         <v>216</v>
@@ -9352,7 +9352,7 @@
         <v>0</v>
       </c>
       <c r="H253" s="3" t="n">
-        <v>173</v>
+        <v>263</v>
       </c>
       <c r="I253" s="3" t="n">
         <v>260</v>
@@ -9387,7 +9387,7 @@
         <v>0</v>
       </c>
       <c r="H254" s="3" t="n">
-        <v>267</v>
+        <v>158</v>
       </c>
       <c r="I254" s="3" t="inlineStr"/>
     </row>
@@ -9420,7 +9420,7 @@
         <v>0</v>
       </c>
       <c r="H255" s="3" t="n">
-        <v>177</v>
+        <v>267</v>
       </c>
       <c r="I255" s="3" t="n">
         <v>272</v>
@@ -9455,7 +9455,7 @@
         <v>0</v>
       </c>
       <c r="H256" s="3" t="n">
-        <v>258</v>
+        <v>165</v>
       </c>
       <c r="I256" s="3" t="inlineStr"/>
     </row>
@@ -9488,7 +9488,7 @@
         <v>0</v>
       </c>
       <c r="H257" s="3" t="n">
-        <v>260</v>
+        <v>163</v>
       </c>
       <c r="I257" s="3" t="n">
         <v>280</v>
@@ -9523,7 +9523,7 @@
         <v>0</v>
       </c>
       <c r="H258" s="3" t="n">
-        <v>171</v>
+        <v>261</v>
       </c>
       <c r="I258" s="3" t="n">
         <v>265</v>
@@ -9558,7 +9558,7 @@
         <v>0</v>
       </c>
       <c r="H259" s="3" t="n">
-        <v>268</v>
+        <v>159</v>
       </c>
       <c r="I259" s="3" t="inlineStr"/>
     </row>
@@ -9591,7 +9591,7 @@
         <v>0</v>
       </c>
       <c r="H260" s="3" t="n">
-        <v>158</v>
+        <v>248</v>
       </c>
       <c r="I260" s="3" t="inlineStr"/>
     </row>
@@ -9657,7 +9657,7 @@
         <v>0</v>
       </c>
       <c r="H262" s="3" t="n">
-        <v>170</v>
+        <v>260</v>
       </c>
       <c r="I262" s="3" t="n">
         <v>251</v>
@@ -9692,7 +9692,7 @@
         <v>0</v>
       </c>
       <c r="H263" s="3" t="n">
-        <v>266</v>
+        <v>157</v>
       </c>
       <c r="I263" s="3" t="inlineStr"/>
     </row>
@@ -9725,7 +9725,7 @@
         <v>0</v>
       </c>
       <c r="H264" s="3" t="n">
-        <v>270</v>
+        <v>161</v>
       </c>
       <c r="I264" s="3" t="inlineStr"/>
     </row>
@@ -9758,7 +9758,7 @@
         <v>0</v>
       </c>
       <c r="H265" s="3" t="n">
-        <v>157</v>
+        <v>247</v>
       </c>
       <c r="I265" s="3" t="n">
         <v>282</v>
@@ -9793,7 +9793,7 @@
         <v>0</v>
       </c>
       <c r="H266" s="3" t="n">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="I266" s="3" t="n">
         <v>225</v>
@@ -9828,7 +9828,7 @@
         <v>0</v>
       </c>
       <c r="H267" s="3" t="n">
-        <v>159</v>
+        <v>250</v>
       </c>
       <c r="I267" s="3" t="inlineStr"/>
     </row>
@@ -9861,7 +9861,7 @@
         <v>0</v>
       </c>
       <c r="H268" s="3" t="n">
-        <v>252</v>
+        <v>236</v>
       </c>
       <c r="I268" s="3" t="n">
         <v>242</v>
@@ -9896,7 +9896,7 @@
         <v>0</v>
       </c>
       <c r="H269" s="3" t="n">
-        <v>265</v>
+        <v>156</v>
       </c>
       <c r="I269" s="3" t="n">
         <v>270</v>
@@ -9931,7 +9931,7 @@
         <v>0</v>
       </c>
       <c r="H270" s="3" t="n">
-        <v>174</v>
+        <v>264</v>
       </c>
       <c r="I270" s="3" t="n">
         <v>268</v>
@@ -9966,7 +9966,7 @@
         <v>0</v>
       </c>
       <c r="H271" s="3" t="n">
-        <v>176</v>
+        <v>266</v>
       </c>
       <c r="I271" s="3" t="n">
         <v>271</v>
@@ -10001,7 +10001,7 @@
         <v>0</v>
       </c>
       <c r="H272" s="3" t="n">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="I272" s="3" t="n">
         <v>212</v>
@@ -10036,7 +10036,7 @@
         <v>0</v>
       </c>
       <c r="H273" s="3" t="n">
-        <v>250</v>
+        <v>234</v>
       </c>
       <c r="I273" s="3" t="n">
         <v>230</v>
@@ -10071,7 +10071,7 @@
         <v>0</v>
       </c>
       <c r="H274" s="3" t="n">
-        <v>262</v>
+        <v>153</v>
       </c>
       <c r="I274" s="3" t="n">
         <v>261</v>

</xml_diff>